<commit_message>
Adding replated resources for Article, Blog and Press release tests with Related Resources links and Exit Disclaimer tests
</commit_message>
<xml_diff>
--- a/test-data/related-resources-data.xlsx
+++ b/test-data/related-resources-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/geopopkh/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC49F85-9468-FF45-AD47-5D34AA847E05}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB1B9D9-36EE-4E49-A3A4-5D663F7C0AFC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="15940" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="15860" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_related_resources" sheetId="1" r:id="rId1"/>
@@ -58,9 +58,6 @@
     <t>Press Release</t>
   </si>
   <si>
-    <t>sharpless-nci-director</t>
-  </si>
-  <si>
     <t>about-cancer/coping/feelings/relaxation/vitamin-d-supplement-cancer-prevention</t>
   </si>
   <si>
@@ -74,6 +71,9 @@
   </si>
   <si>
     <t>news-events/cancer-currents-blog/2019/human-tumor-atlas-network-cancer-maps</t>
+  </si>
+  <si>
+    <t>espanol/noticias/comunicados-de-prensa/2019/aprendizaje-profundo-cancer-cuello-uterino-examenes-de</t>
   </si>
 </sst>
 </file>
@@ -432,7 +432,7 @@
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="74.6640625" customWidth="1"/>
+    <col min="1" max="1" width="83.1640625" customWidth="1"/>
     <col min="2" max="2" width="23.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -460,10 +460,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
         <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -471,10 +471,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -502,6 +502,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="94.6640625" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -528,7 +530,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -539,13 +541,13 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding Related Resources with Exit Disclaimer
</commit_message>
<xml_diff>
--- a/test-data/related-resources-data.xlsx
+++ b/test-data/related-resources-data.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/geopopkh/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB1B9D9-36EE-4E49-A3A4-5D663F7C0AFC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C2C97E-2A9E-6640-B605-0EB222D307B3}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="15860" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
+    <workbookView xWindow="300" yWindow="700" windowWidth="33220" windowHeight="18880" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_related_resources" sheetId="1" r:id="rId1"/>
     <sheet name="pages_without_related_resources" sheetId="2" r:id="rId2"/>
+    <sheet name="pages_with_external_resources" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="20">
   <si>
     <t>path</t>
   </si>
@@ -74,6 +75,18 @@
   </si>
   <si>
     <t>espanol/noticias/comunicados-de-prensa/2019/aprendizaje-profundo-cancer-cuello-uterino-examenes-de</t>
+  </si>
+  <si>
+    <t>sharpless-nci-director</t>
+  </si>
+  <si>
+    <t>expectedExternalCount</t>
+  </si>
+  <si>
+    <t>espanol/cancer/sobrellevar/sentimientos</t>
+  </si>
+  <si>
+    <t>espanol/cancer/sobrellevar/self-image</t>
   </si>
 </sst>
 </file>
@@ -109,12 +122,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,7 +517,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E4A3B0B-8B0F-6546-A344-A90113573E35}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="94.6640625" customWidth="1"/>
@@ -550,6 +569,103 @@
         <v>6</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{559EFC9A-164C-8144-9EB0-75C1F6F01408}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="63.1640625" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="23.5" customWidth="1"/>
+    <col min="5" max="5" width="13.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updating Related resourcess tests to address data Provider name change and comment changes
</commit_message>
<xml_diff>
--- a/test-data/related-resources-data.xlsx
+++ b/test-data/related-resources-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02C2C97E-2A9E-6640-B605-0EB222D307B3}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB253DB-8DA3-C74C-9415-587630FCFCD2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="700" windowWidth="33220" windowHeight="18880" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
+    <workbookView xWindow="3360" yWindow="3400" windowWidth="33220" windowHeight="18880" activeTab="2" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_related_resources" sheetId="1" r:id="rId1"/>
@@ -453,6 +453,7 @@
   <cols>
     <col min="1" max="1" width="83.1640625" customWidth="1"/>
     <col min="2" max="2" width="23.5" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -596,7 +597,7 @@
     <col min="5" max="5" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
updated Related Resources external link check
</commit_message>
<xml_diff>
--- a/test-data/related-resources-data.xlsx
+++ b/test-data/related-resources-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB253DB-8DA3-C74C-9415-587630FCFCD2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7F27DD-8723-3D42-95A6-57DA99318D11}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3360" yWindow="3400" windowWidth="33220" windowHeight="18880" activeTab="2" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16140" activeTab="2" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_related_resources" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="26">
   <si>
     <t>path</t>
   </si>
@@ -87,6 +87,24 @@
   </si>
   <si>
     <t>espanol/cancer/sobrellevar/self-image</t>
+  </si>
+  <si>
+    <t>about-cancer/coping/feelings/relaxation/hpv-vaccine-presidents-cancer-panel-improving-uptake</t>
+  </si>
+  <si>
+    <t>Blog Post</t>
+  </si>
+  <si>
+    <t>about-cancer/coping/feelings/relaxation/duke-university</t>
+  </si>
+  <si>
+    <t>Cancer Center</t>
+  </si>
+  <si>
+    <t>about-cancer/coping/feelings/relaxation/loukissas-jen-biography</t>
+  </si>
+  <si>
+    <t>Biography</t>
   </si>
 </sst>
 </file>
@@ -483,10 +501,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -497,7 +515,7 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -505,10 +523,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -588,10 +606,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{559EFC9A-164C-8144-9EB0-75C1F6F01408}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="63.1640625" customWidth="1"/>
+    <col min="1" max="1" width="82.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.1640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="23.5" customWidth="1"/>
     <col min="5" max="5" width="13.5" customWidth="1"/>
@@ -667,6 +685,62 @@
         <v>6</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="3">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated RR test and  data for missing files on dev
</commit_message>
<xml_diff>
--- a/test-data/related-resources-data.xlsx
+++ b/test-data/related-resources-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7F27DD-8723-3D42-95A6-57DA99318D11}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B343591C-1F21-C841-986A-948E7B521A93}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16140" activeTab="2" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
+    <workbookView xWindow="4280" yWindow="2760" windowWidth="28800" windowHeight="16140" activeTab="1" xr2:uid="{112BCE41-1B7B-AF44-BEF2-07A92CFC037C}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_related_resources" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="26">
   <si>
     <t>path</t>
   </si>
@@ -59,27 +59,18 @@
     <t>Press Release</t>
   </si>
   <si>
-    <t>about-cancer/coping/feelings/relaxation/vitamin-d-supplement-cancer-prevention</t>
-  </si>
-  <si>
     <t>Blog Page</t>
   </si>
   <si>
     <t>news-events/press-releases/2018/oropharyngeal-hpv-cisplatin</t>
   </si>
   <si>
-    <t>espanol/about-cancer/coping/feelings/relaxation/vitamina-d-complemento-cancer-prevencion</t>
-  </si>
-  <si>
     <t>news-events/cancer-currents-blog/2019/human-tumor-atlas-network-cancer-maps</t>
   </si>
   <si>
     <t>espanol/noticias/comunicados-de-prensa/2019/aprendizaje-profundo-cancer-cuello-uterino-examenes-de</t>
   </si>
   <si>
-    <t>sharpless-nci-director</t>
-  </si>
-  <si>
     <t>expectedExternalCount</t>
   </si>
   <si>
@@ -89,9 +80,6 @@
     <t>espanol/cancer/sobrellevar/self-image</t>
   </si>
   <si>
-    <t>about-cancer/coping/feelings/relaxation/hpv-vaccine-presidents-cancer-panel-improving-uptake</t>
-  </si>
-  <si>
     <t>Blog Post</t>
   </si>
   <si>
@@ -105,6 +93,18 @@
   </si>
   <si>
     <t>Biography</t>
+  </si>
+  <si>
+    <t>news-events/cancer-currents-blog/2019/hpv-vaccine-presidents-cancer-panel-improving-uptake</t>
+  </si>
+  <si>
+    <t>news-events/cancer-currents-blog/2019/vitamin-d-supplement-cancer-prevention</t>
+  </si>
+  <si>
+    <t>espanol/node/116/2019/vitamina-d-complemento-cancer-prevencion</t>
+  </si>
+  <si>
+    <t>news-events/press-releases/2019/deep-learning-cervical-cancer-screening</t>
   </si>
 </sst>
 </file>
@@ -466,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ABDEF67-3BF3-604C-97A8-A43819B8E79D}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="83.1640625" customWidth="1"/>
@@ -498,7 +498,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -509,24 +509,57 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
-        <v>6</v>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -568,7 +601,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -579,7 +612,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -590,7 +623,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -620,7 +653,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -631,7 +664,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="3">
         <v>3</v>
@@ -659,7 +692,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B4" s="3">
         <v>1</v>
@@ -673,7 +706,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B5" s="3">
         <v>0</v>
@@ -687,13 +720,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6" s="3">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
@@ -701,13 +734,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B7" s="3">
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
@@ -715,13 +748,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B8" s="3">
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
@@ -729,13 +762,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="B9" s="3">
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
         <v>6</v>

</xml_diff>